<commit_message>
Vigilancia 2026-10-02 07:33 UTC
</commit_message>
<xml_diff>
--- a/docs/informes/edistribucion_demanda_2026-09-03.xlsx
+++ b/docs/informes/edistribucion_demanda_2026-09-03.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Incrementos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Afloramientos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Incrementos" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Incrementos'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Afloramientos'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Incrementos'!$A$1:$I$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +480,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>03/08/2026  (https://www.edistribucion.com/content/dam/edistribucion/conexion-a-la-red/descargables/nodos/demanda/202608/2026_08_03_R1299_demanda.csv)</t>
+          <t>02/10/2026  (https://www.edistribucion.com/content/dam/edistribucion/conexion-a-la-red/descargables/nodos/demanda/202610/2026_10_02_R1299_demanda.csv)</t>
         </is>
       </c>
     </row>
@@ -512,7 +514,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>30/09/2026 10:08</t>
+          <t>02/10/2026 09:33</t>
         </is>
       </c>
     </row>
@@ -527,7 +529,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -537,7 +539,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -591,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -655,7 +657,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MONCAYO 45 kV</t>
+          <t>S.C.OLORDE 25 kV</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -664,35 +666,39 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>40.07</v>
+        <v>11.34</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>39.07</v>
+        <v>11.34</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>07 - C.León</t>
+          <t>09 - Catalunya</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Soria</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Ólvega</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Capacidad que podría no estar disponible en su totalidad, en función de la explotación de sus barras. A determinar en estudio individual.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>LA_LOMA 45 kV</t>
+          <t>BESOS 25 kV</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -701,152 +707,184 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>30</v>
+        <v>2.15</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>29</v>
+        <v>2.15</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>07 - C.León</t>
+          <t>09 - Catalunya</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Soria</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Ólvega</t>
+          <t>Sant Adrià de Besòs</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>S_MADERO 45 kV</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+  </sheetData>
+  <autoFilter ref="A1:I3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Nudo</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Capacidad</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Antes (MW)</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Ahora (MW)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Variación (MW)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Comunidad Autónoma</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Provincia</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Municipio</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>VIC 132 kV</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Capacidad firme disponible (MW)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>07 - C.León</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Soria</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Ólvega</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="C2" s="4" t="n">
+        <v>47.24</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>96.63</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>49.39</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>09 - Catalunya</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Vic</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>S.COLOMA 25 kV</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Capacidad firme disponible (MW)</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>9.66</v>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="C3" s="4" t="n">
+        <v>14.98</v>
+      </c>
+      <c r="D3" s="4" t="n">
         <v>29.33</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>19.67</v>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E3" s="4" t="n">
+        <v>14.35</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>09 - Catalunya</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Barcelona</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Santa Coloma de Gramenet</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Capacidad que podría no estar disponible en su totalidad, en función de la explotación de sus barras. A determinar en estudio individual.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>JUNEDA 25 kV</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Capacidad firme disponible (MW)</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>9.960000000000001</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>28.94</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>18.98</v>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>09 - Catalunya</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Lleida</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Juneda</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Subestación con espacio insuficiente o posibles restricciones para su ampliación. Dificultad para la conexión de una nueva posición o con coste muy elevado.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
+  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>